<commit_message>
Implement OOP structure for PC components and animal classes
- Added Vifte class to represent a fan component with attributes like size, RPM, airflow, noise level, and connection type.
- Created Dyr class as a base for different animal types, including methods for presenting and aging.
- Developed subclasses for specific animals: Hund, Katt, Fugl, Slange, Hest, and Fisk, each with unique attributes and behaviors.
- Introduced Ansatt and Leder classes for employee management, with methods for salary calculation and output.
- Implemented Person class as a base for employee details, including methods for salary calculation over 12 months.
- Added functionality to calculate monthly salary and print employee details.
- Created scripts to instantiate and manage employee objects, demonstrating the use of the classes.
</commit_message>
<xml_diff>
--- a/02-oppgaver/10-crm_system/11-crm_testdata.xlsx
+++ b/02-oppgaver/10-crm_system/11-crm_testdata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://telemarkfylke.sharepoint.com/sites/Section_2526-POV-13163348/Delte dokumenter/General/03-Elevarbeid-25/William/02-oppgaver/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://telemarkfylke.sharepoint.com/sites/Section_2526-POV-13163348/Delte dokumenter/General/03-Elevarbeid-25/William/02-oppgaver/10-crm_system/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="154" documentId="8_{1D13375F-92DB-4F39-BD2F-CDD0796A3D0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AE9B03D-2FA3-4E76-8652-C9B1F3ED7F5F}"/>
+  <xr:revisionPtr revIDLastSave="164" documentId="8_{1D13375F-92DB-4F39-BD2F-CDD0796A3D0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{537F8D99-6EB7-4DD5-97DA-8ACF7D56E224}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F8A5777D-2C86-46AE-9F01-07F9D4B63122}"/>
+    <workbookView minimized="1" xWindow="-105" yWindow="3060" windowWidth="12105" windowHeight="5940" xr2:uid="{F8A5777D-2C86-46AE-9F01-07F9D4B63122}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="47">
   <si>
     <t>Kunde</t>
   </si>
@@ -171,6 +171,12 @@
   </si>
   <si>
     <t>bergen</t>
+  </si>
+  <si>
+    <t>kunde</t>
+  </si>
+  <si>
+    <t>ansatt</t>
   </si>
 </sst>
 </file>
@@ -300,9 +306,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>3840</xdr:colOff>
+      <xdr:colOff>7015</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>125760</xdr:rowOff>
+      <xdr:rowOff>122585</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
       <mc:Choice Requires="xdr14">
@@ -430,7 +436,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>28680</xdr:colOff>
+      <xdr:colOff>25505</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>95700</xdr:rowOff>
     </xdr:to>
@@ -512,7 +518,7 @@
       <inkml:brushProperty name="height" value="0.035" units="cm"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1407 4 24575,'-67'-1'0,"30"-1"0,0 2 0,0 1 0,0 2 0,1 1 0,-1 2 0,-42 13 0,62-11 0,-1 1 0,2 1 0,-1 1 0,1 0 0,1 1 0,-22 21 0,-5 4 0,24-23 0,0 1 0,2 0 0,0 1 0,1 1 0,0 1 0,1 0 0,1 0 0,1 2 0,1-1 0,-11 29 0,-28 59 0,30-67 0,-16 47 0,-1 4 0,-7 24 0,19-33 0,-65 248 0,49-183 0,27-108 0,3 2 0,1-1 0,2 1 0,-5 58 0,12-60 0,-2 1 0,-2-1 0,-1-1 0,-2 1 0,-2-1 0,-1-1 0,-2 0 0,-2 0 0,-24 42 0,21-47 0,-94 189 0,102-196 0,0 2 0,2-1 0,1 1 0,2 1 0,0-1 0,-1 53 0,6-75 0,0 15 0,0 0 0,6 31 0,-5-43 0,1-1 0,0 1 0,1-1 0,0 0 0,0 0 0,1 0 0,0 0 0,0-1 0,10 13 0,30 29 0,-29-33 0,-1 1 0,0 0 0,-1 1 0,-1 1 0,20 36 0,-5 12 0,-3 1 0,17 73 0,-27-82 0,-2 1 0,3 62 0,-11-95 0,0 1 0,13 38 0,-10-41 0,-1 2 0,0-1 0,1 29 0,-6-20 0,1 1 0,2 0 0,2 0 0,1-1 0,15 45 0,34 52 0,121 203 0,-80-159 0,-84-150 0,1 0 0,1-1 0,1-1 0,2 0 0,0-1 0,1-1 0,1-1 0,1-1 0,40 29 0,188 110 0,-210-129 0,46 46 0,-54-46 0,1-2 0,51 34 0,-21-27 0,1-3 0,1-3 0,2-3 0,0-3 0,2-3 0,96 16 0,-94-27 0,0-3 0,129-7 0,-62-1 0,446 3 0,-573 0 0,-1 0 0,1 0 0,-1-1 0,0-1 0,1 1 0,-1-2 0,0 1 0,0-1 0,0 0 0,0-1 0,-1 0 0,1-1 0,-1 1 0,0-2 0,-1 1 0,1-1 0,12-13 0,8-7 0,-9 8 0,0-1 0,30-39 0,-38 43 0,1 2 0,1 0 0,0 1 0,0 0 0,1 0 0,20-11 0,-13 9 0,36-33 0,-50 40 0,0 0 0,-1 0 0,-1-1 0,1 0 0,-1 0 0,0 0 0,-1-1 0,7-17 0,-8 17 0,0 0 0,1 0 0,0 0 0,0 1 0,1 0 0,0-1 0,7-7 0,-8 12 0,0-1 0,1 1 0,-1 1 0,1-1 0,0 1 0,0 0 0,0 0 0,1 0 0,-1 0 0,1 1 0,-1 0 0,11-2 0,16-3-1365,-3 0-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1407 4 24575,'-67'-1'0,"30"-1"0,0 2 0,0 1 0,0 2 0,1 1 0,-1 1 0,-42 13 0,62-10 0,-1 1 0,2 0 0,-1 2 0,1-1 0,1 2 0,-22 19 0,-5 5 0,24-23 0,0 1 0,2 0 0,0 2 0,1 0 0,0 1 0,1 0 0,1 1 0,1 1 0,1-1 0,-11 28 0,-28 56 0,30-64 0,-16 45 0,-1 4 0,-7 22 0,19-30 0,-65 236 0,49-175 0,27-103 0,3 2 0,1-1 0,2 2 0,-5 54 0,12-57 0,-2 1 0,-2 0 0,-1-2 0,-2 1 0,-2-1 0,-1 0 0,-2-1 0,-2 0 0,-24 41 0,21-46 0,-94 181 0,102-187 0,0 2 0,2-1 0,1 0 0,2 2 0,0-1 0,-1 50 0,6-71 0,0 14 0,0 0 0,6 30 0,-5-42 0,1 0 0,0 1 0,1-2 0,0 1 0,0 0 0,1-1 0,0 1 0,0-1 0,10 12 0,30 28 0,-29-32 0,-1 1 0,0 1 0,-1 0 0,-1 1 0,20 35 0,-5 11 0,-3 1 0,17 69 0,-27-78 0,-2 2 0,3 58 0,-11-90 0,0 1 0,13 36 0,-10-39 0,-1 2 0,0-2 0,1 29 0,-6-20 0,1 2 0,2-1 0,2 1 0,1-2 0,15 43 0,34 50 0,121 194 0,-80-152 0,-84-143 0,1 0 0,1-1 0,1-1 0,2 0 0,0-1 0,1-1 0,1-1 0,1-1 0,40 28 0,188 105 0,-210-124 0,46 45 0,-54-44 0,1-3 0,51 34 0,-21-27 0,1-2 0,1-4 0,2-2 0,0-3 0,2-3 0,96 16 0,-94-27 0,0-2 0,129-7 0,-62-1 0,446 3 0,-573 0 0,-1 0 0,1 0 0,-1-1 0,0-1 0,1 1 0,-1-1 0,0 0 0,0-1 0,0 0 0,0-1 0,-1 0 0,1 0 0,-1 0 0,0-2 0,-1 1 0,1 0 0,12-14 0,8-5 0,-9 6 0,0 0 0,30-37 0,-38 41 0,1 1 0,1 1 0,0 0 0,0 1 0,1-1 0,20-10 0,-13 9 0,36-32 0,-50 39 0,0-1 0,-1 0 0,-1 0 0,1-1 0,-1 0 0,0 1 0,-1-2 0,7-16 0,-8 17 0,0-1 0,1 1 0,0-1 0,0 1 0,1 1 0,0-2 0,7-6 0,-8 11 0,0-1 0,1 1 0,-1 2 0,1-2 0,0 1 0,0 0 0,0 0 0,1 0 0,-1 0 0,1 1 0,-1 1 0,11-3 0,16-3-1365,-3 0-5461</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -540,7 +546,7 @@
       <inkml:brushProperty name="color" value="#E71224"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">3469 5290 24575,'0'0'0,"0"0"0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1-1 0,-1 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,-1 0 0,-7-13 0,-15-10 0,-15-3 0,-1 1 0,-1 2 0,-1 3 0,-1 1 0,-60-19 0,-136-31 0,138 33 0,2-5 0,1-5 0,-99-63 0,152 81 0,-153-110 0,176 121 0,1-2 0,0-1 0,1 0 0,1-2 0,1 0 0,-23-38 0,4-7 0,16 26 0,-3 0 0,-1 2 0,-1 1 0,-3 0 0,-33-34 0,-122-90 0,4 4 0,-482-521 0,637 652 0,-1 3 0,2-1 0,1-2 0,1 0 0,1-1 0,-31-58 0,47 72 0,1 1 0,0-1 0,0 1 0,2-1 0,-1 0 0,2 0 0,0 0 0,2-14 0,-1 12 0,-1-1 0,0 0 0,-1 0 0,-6-28 0,-2 16 0,-2 2 0,-1-1 0,-2 1 0,0 1 0,-34-46 0,-10-17 0,42 61 0,-27-44 0,3-2 0,3-1 0,-28-86 0,17 41 0,34 89 0,0-1 0,2 0 0,-10-47 0,-18-71 0,28 112 0,1 0 0,2 0 0,2-1 0,-4-65 0,14-335 0,-3 424 0,2 1 0,0-1 0,0 1 0,1 0 0,1-1 0,1 2 0,0-1 0,0 0 0,2 1 0,11-20 0,-7 17 0,1-1 0,1 1 0,0 1 0,0 0 0,2 1 0,0 1 0,19-14 0,146-77 0,-68 42 0,175-102 0,-275 157 0,-1 0 0,0 0 0,0 0 0,1 2 0,0-1 0,0 1 0,0 1 0,1 0 0,-1 1 0,1 0 0,23-1 0,8 1 0,-1-3 0,44-10 0,-45 7 0,0 2 0,53-2 0,-55 7 0,44-9-1,-35 4-1363,-23 3-5462</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">3461 5060 24575,'0'0'0,"0"0"0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1-1 0,-1 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,-1 0 0,-7-12 0,-15-10 0,-15-3 0,-1 1 0,-1 2 0,-1 3 0,0 1 0,-61-19 0,-136-29 0,139 32 0,1-5 0,1-5 0,-99-60 0,153 77 0,-154-105 0,176 115 0,1-1 0,0-1 0,1 0 0,1-2 0,1 0 0,-23-36 0,4-8 0,16 26 0,-2 0 0,-2 2 0,-1 0 0,-3 1 0,-33-33 0,-122-86 0,5 4 0,-482-498 0,636 623 0,-1 3 0,2-1 0,1-2 0,1 0 0,2-1 0,-32-55 0,47 69 0,1 0 0,0 0 0,0 1 0,2-2 0,-1 1 0,2-1 0,0 1 0,2-14 0,-1 12 0,-1-1 0,0-1 0,-1 1 0,-6-27 0,-2 15 0,-2 2 0,-1 0 0,-2 0 0,0 1 0,-34-44 0,-10-16 0,42 58 0,-27-42 0,3-1 0,3-2 0,-27-82 0,16 39 0,34 85 0,0 0 0,2-1 0,-10-44 0,-18-69 0,28 108 0,1-1 0,2 1 0,2-1 0,-4-63 0,14-320 0,-3 406 0,2 1 0,0-2 0,0 2 0,1 0 0,1-2 0,1 3 0,0-2 0,0 1 0,2 1 0,11-20 0,-7 17 0,1-2 0,1 2 0,0 1 0,0-1 0,2 2 0,0 1 0,19-14 0,145-74 0,-67 41 0,174-98 0,-274 150 0,-1 1 0,0-1 0,0 0 0,1 3 0,0-2 0,0 1 0,0 1 0,1 0 0,-1 1 0,1 1 0,23-2 0,8 1 0,-1-3 0,43-9 0,-44 6 0,0 3 0,53-3 0,-55 7 0,44-8-1,-35 3-1363,-23 3-5462</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -568,7 +574,7 @@
       <inkml:brushProperty name="color" value="#33CCFF"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">3417 4236 24575,'-1'1'0,"0"0"0,1 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,0-1 0,0 1 0,-1-1 0,1 0 0,0 0 0,-1 1 0,1-1 0,-2 0 0,-39 6 0,39-6 0,-25 3 0,0-2 0,0-1 0,0-1 0,0-2 0,0 0 0,1-2 0,-1-1 0,1-1 0,-34-15 0,-38-15 0,-112-25 0,-94-23 0,81 16 0,98 28 0,-268-94 0,281 89 0,-151-86 0,259 129 0,-46-25 0,1-3 0,2-1 0,-68-59 0,-47-72 0,-19-18 0,158 161 0,2-1 0,1 0 0,0-2 0,2-1 0,0 0 0,2-1 0,1-1 0,-21-43 0,16 24 0,-3 1 0,-54-76 0,14 24 0,-13-20 0,46 74 0,3-1 0,1-1 0,-36-84 0,57 110 0,2 0 0,1-1 0,0 1 0,1-1 0,1 1 0,2-38 0,0 33 0,0 0 0,-2-1 0,-8-42 0,-5 4 0,2 0 0,3-1 0,-1-85 0,9 3 0,5-179 0,1 279 0,1-1 0,23-82 0,42-83 0,-49 148 0,-12 39 0,1-1 0,1 2 0,1 0 0,1 0 0,1 1 0,1 1 0,1 0 0,20-18 0,-13 15 0,2 1 0,1 2 0,1 0 0,0 2 0,54-26 0,-35 25 0,1 3 0,0 2 0,1 3 0,1 1 0,0 3 0,98-5 0,-89 12 0,-27 2 0,-1-2 0,1-1 0,-1-2 0,57-14 0,-48 5-227,0 1-1,0 3 1,1 1-1,0 2 1,63-1-1,-73 7-6598</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">3408 4045 24575,'-1'1'0,"0"0"0,1 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,0-1 0,0 1 0,-1-1 0,1 0 0,0 0 0,-1 0 0,1 0 0,-2 0 0,-39 6 0,39-6 0,-25 3 0,0-2 0,0-1 0,0-1 0,1-2 0,-1 0 0,1-1 0,-1-2 0,1-1 0,-34-14 0,-38-14 0,-111-24 0,-94-23 0,80 17 0,99 25 0,-268-89 0,280 86 0,-150-84 0,258 125 0,-46-25 0,1-3 0,2 0 0,-68-57 0,-46-69 0,-20-17 0,158 154 0,2-1 0,1 0 0,0-2 0,2-1 0,1 0 0,1-1 0,1 0 0,-21-42 0,16 23 0,-3 1 0,-54-73 0,14 23 0,-13-18 0,46 70 0,4-2 0,0 0 0,-36-80 0,57 105 0,2 0 0,1-1 0,0 1 0,1-2 0,1 2 0,2-36 0,0 31 0,0 0 0,-2-1 0,-8-40 0,-5 4 0,2-1 0,3 0 0,-1-81 0,9 2 0,5-170 0,1 266 0,1-1 0,23-78 0,42-80 0,-49 142 0,-12 37 0,1-1 0,1 2 0,1 1 0,0-1 0,2 1 0,1 0 0,1 1 0,20-17 0,-13 14 0,2 1 0,1 2 0,1 0 0,0 2 0,54-25 0,-35 24 0,0 3 0,1 1 0,1 4 0,1 0 0,0 4 0,98-6 0,-90 12 0,-26 2 0,-1-2 0,1 0 0,-1-3 0,57-13 0,-48 4-227,0 2-1,-1 2 1,2 1-1,0 3 1,63-2-1,-73 7-6598</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -890,19 +896,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{894EEB08-6815-454F-A204-08D3D9480ADE}">
   <dimension ref="B3:M36"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="24.42578125" customWidth="1"/>
+    <col min="3" max="3" width="24.453125" customWidth="1"/>
     <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.54296875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
         <v>0</v>
       </c>
@@ -912,7 +918,7 @@
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
     </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>12</v>
       </c>
@@ -938,7 +944,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B5" s="6">
         <v>1</v>
       </c>
@@ -964,7 +970,7 @@
         <v>234343453</v>
       </c>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B6" s="6">
         <v>2</v>
       </c>
@@ -990,7 +996,7 @@
         <v>234765453</v>
       </c>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B7" s="6">
         <v>3</v>
       </c>
@@ -1016,18 +1022,18 @@
         <v>919758142</v>
       </c>
     </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:13" x14ac:dyDescent="0.35">
       <c r="F8" s="2"/>
     </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:13" x14ac:dyDescent="0.35">
       <c r="F9" s="2"/>
     </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:13" x14ac:dyDescent="0.35">
       <c r="C12" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:13" x14ac:dyDescent="0.35">
       <c r="C13" s="5" t="s">
         <v>17</v>
       </c>
@@ -1062,7 +1068,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:13" x14ac:dyDescent="0.35">
       <c r="C14" s="6">
         <v>1</v>
       </c>
@@ -1097,7 +1103,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:13" x14ac:dyDescent="0.35">
       <c r="C15" s="6">
         <v>2</v>
       </c>
@@ -1132,7 +1138,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:13" x14ac:dyDescent="0.35">
       <c r="C16" s="6">
         <v>3</v>
       </c>
@@ -1167,64 +1173,94 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="3:6" x14ac:dyDescent="0.35">
       <c r="F17" s="2"/>
     </row>
-    <row r="18" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:6" x14ac:dyDescent="0.35">
       <c r="F18" s="2"/>
     </row>
-    <row r="19" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:6" x14ac:dyDescent="0.35">
       <c r="F19" s="2"/>
     </row>
-    <row r="20" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:6" x14ac:dyDescent="0.35">
+      <c r="C20" t="s">
+        <v>45</v>
+      </c>
+      <c r="D20" t="s">
+        <v>46</v>
+      </c>
       <c r="F20" s="2"/>
     </row>
-    <row r="21" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:6" x14ac:dyDescent="0.35">
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21">
+        <v>2</v>
+      </c>
       <c r="F21" s="2"/>
     </row>
-    <row r="22" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:6" x14ac:dyDescent="0.35">
+      <c r="C22">
+        <v>2</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
       <c r="F22" s="2"/>
     </row>
-    <row r="23" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:6" x14ac:dyDescent="0.35">
+      <c r="C23">
+        <v>2</v>
+      </c>
+      <c r="D23">
+        <v>2</v>
+      </c>
       <c r="F23" s="2"/>
     </row>
-    <row r="24" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:6" x14ac:dyDescent="0.35">
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24">
+        <v>2</v>
+      </c>
       <c r="F24" s="2"/>
     </row>
-    <row r="25" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:6" x14ac:dyDescent="0.35">
       <c r="F25" s="2"/>
     </row>
-    <row r="26" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="3:6" x14ac:dyDescent="0.35">
       <c r="F26" s="2"/>
     </row>
-    <row r="27" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:6" x14ac:dyDescent="0.35">
       <c r="F27" s="2"/>
     </row>
-    <row r="28" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:6" x14ac:dyDescent="0.35">
       <c r="F28" s="2"/>
     </row>
-    <row r="29" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="3:6" x14ac:dyDescent="0.35">
       <c r="F29" s="2"/>
     </row>
-    <row r="30" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:6" x14ac:dyDescent="0.35">
       <c r="F30" s="2"/>
     </row>
-    <row r="31" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="3:6" x14ac:dyDescent="0.35">
       <c r="F31" s="2"/>
     </row>
-    <row r="32" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:6" x14ac:dyDescent="0.35">
       <c r="F32" s="2"/>
     </row>
-    <row r="33" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F33" s="2"/>
     </row>
-    <row r="34" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F34" s="2"/>
     </row>
-    <row r="35" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F35" s="2"/>
     </row>
-    <row r="36" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F36" s="2"/>
     </row>
   </sheetData>
@@ -1243,28 +1279,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="0303f316-29c9-46e3-af50-1b05a60d057b" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6c201026-1728-48f4-a932-5852b16e16b0">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100D440BF34C7EEB746A2B04D9352B0A354" ma:contentTypeVersion="10" ma:contentTypeDescription="Opprett et nytt dokument." ma:contentTypeScope="" ma:versionID="b1d27b81dc11b1c2fd8d3a42c9c73486">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6c201026-1728-48f4-a932-5852b16e16b0" xmlns:ns3="0303f316-29c9-46e3-af50-1b05a60d057b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b9cca73293918ec8e86f994d897458cd" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100D440BF34C7EEB746A2B04D9352B0A354" ma:contentTypeVersion="10" ma:contentTypeDescription="Opprett et nytt dokument." ma:contentTypeScope="" ma:versionID="6347883b1269eaddd3cd32f0c0cac89c">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6c201026-1728-48f4-a932-5852b16e16b0" xmlns:ns3="0303f316-29c9-46e3-af50-1b05a60d057b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cf2cb6a01f64d6e6f29ab99dd9af0f53" ns2:_="" ns3:_="">
     <xsd:import namespace="6c201026-1728-48f4-a932-5852b16e16b0"/>
     <xsd:import namespace="0303f316-29c9-46e3-af50-1b05a60d057b"/>
     <xsd:element name="properties">
@@ -1451,15 +1467,28 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="0303f316-29c9-46e3-af50-1b05a60d057b" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6c201026-1728-48f4-a932-5852b16e16b0">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E108DD08-0B53-495B-91B8-D64E9E1CBCA9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0303f316-29c9-46e3-af50-1b05a60d057b"/>
-    <ds:schemaRef ds:uri="6c201026-1728-48f4-a932-5852b16e16b0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76871C77-9878-4B53-A7AA-EF13DEB7A5F1}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1471,20 +1500,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0205E525-28AA-47E8-9424-2DA036C0C059}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E108DD08-0B53-495B-91B8-D64E9E1CBCA9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0303f316-29c9-46e3-af50-1b05a60d057b"/>
     <ds:schemaRef ds:uri="6c201026-1728-48f4-a932-5852b16e16b0"/>
-    <ds:schemaRef ds:uri="0303f316-29c9-46e3-af50-1b05a60d057b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>